<commit_message>
Maps: Esri World Street Map for the Map view (OSM tiles refuse local-file pages and business use); docs updated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvztMCDJjkzUV6LkhkyE5H
</commit_message>
<xml_diff>
--- a/ls-attendance-tracker/docs/LS Attendance - Azure Resource Requirements.xlsx
+++ b/ls-attendance-tracker/docs/LS Attendance - Azure Resource Requirements.xlsx
@@ -2314,7 +2314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2384,12 +2384,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>tile.openstreetmap.org</t>
+          <t>server.arcgisonline.com</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Map view tiles</t>
+          <t>Map view (Esri World Street Map), Satellite view (World Imagery) + place labels</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -2399,41 +2399,41 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>OSM tile usage policy: light use; attribution shown</t>
+          <t>Esri basemap terms; attribution shown</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>server.arcgisonline.com</t>
+          <t>photon.komoot.io</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Satellite view (Esri World Imagery) + place labels</t>
+          <t>Place search type-ahead</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Esri basemap terms; attribution shown</t>
+          <t>Free OSM-based service, fair use</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>photon.komoot.io</t>
+          <t>nominatim.openstreetmap.org</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Place search type-ahead</t>
+          <t>Place search on Enter</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -2443,19 +2443,19 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Free OSM-based service, fair use</t>
+          <t>Nominatim usage policy: max 1 request/second</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>nominatim.openstreetmap.org</t>
+          <t>geocode-api.arcgis.com</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Place search on Enter</t>
+          <t>ArcGIS search (only when a key is set)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -2464,28 +2464,6 @@
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Nominatim usage policy: max 1 request/second</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>geocode-api.arcgis.com</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>ArcGIS search (only when a key is set)</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>ArcGIS Location Platform, per request</t>
         </is>
@@ -2816,7 +2794,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Maps, zones, pins</t>
+          <t>Maps (Esri street + satellite tiles), zones, pins</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Invoice pack: project documents (WOI uploaded once per project), PDF page identification with thumbnails and field extraction, uploaded SAP page and signed timesheets per invoice, one-click pack PDF; documents kept in IndexedDB and in backups
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvztMCDJjkzUV6LkhkyE5H
</commit_message>
<xml_diff>
--- a/ls-attendance-tracker/docs/LS Attendance - Azure Resource Requirements.xlsx
+++ b/ls-attendance-tracker/docs/LS Attendance - Azure Resource Requirements.xlsx
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Leaflet 1.9.4, SheetJS 0.18.5, ExcelJS 4.4.0, pdf-lib 1.17.1, qrcode-generator 1.4.4</t>
+          <t>Leaflet 1.9.4, SheetJS 0.18.5, ExcelJS 4.4.0, pdf-lib 1.17.1, pdf.js 4.10.38, html2canvas 1.4.1, qrcode-generator 1.4.4</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -2481,7 +2481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Merge PDFs into the invoice pack</t>
+          <t>Build the invoice pack PDF (copy uploaded pages, place generated pages)</t>
         </is>
       </c>
     </row>
@@ -2887,12 +2887,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>qrcode-generator</t>
+          <t>pdf.js (pdfjs-dist)</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>1.4.4</t>
+          <t>4.10.38</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -2902,142 +2902,142 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>QR code on PIN slips</t>
+          <t>Read uploaded PDFs: page text and thumbnails for page identification</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Browser storage</t>
+          <t>Front end</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>IndexedDB, localStorage, Service Worker</t>
+          <t>html2canvas</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Built-in</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Browser</t>
+          <t>cdn.jsdelivr.net</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Admin data, offline punch queue, remembered Emp ID</t>
+          <t>Render generated break-up and timesheet pages to images for the pack</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Supported browsers</t>
+          <t>Front end</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Edge / Chrome (admin)</t>
+          <t>qrcode-generator</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Current, Chromium 110+</t>
+          <t>1.4.4</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>cdn.jsdelivr.net</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Printing uses the browser print dialog</t>
+          <t>QR code on PIN slips</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Supported browsers</t>
+          <t>Browser storage</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Chrome for Android / Safari on iOS (worker)</t>
+          <t>IndexedDB, localStorage, Service Worker</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Android 9+ Chrome 110+; iOS 16.4+</t>
+          <t>Built-in</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Browser</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Camera and GPS need HTTPS; add to Home screen</t>
+          <t>Admin data, offline punch queue, remembered Emp ID</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Build / test</t>
+          <t>Supported browsers</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Node.js</t>
+          <t>Edge / Chrome (admin)</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>20+ (tested 22.22)</t>
+          <t>Current, Chromium 110+</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Developer PC / CI</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>node build.mjs; tests in tests/</t>
+          <t>Printing uses the browser print dialog</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Build / test</t>
+          <t>Supported browsers</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Playwright + Chromium</t>
+          <t>Chrome for Android / Safari on iOS (worker)</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>1.47+</t>
+          <t>Android 9+ Chrome 110+; iOS 16.4+</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>End-to-end tests with fake GPS and camera</t>
+          <t>Camera and GPS need HTTPS; add to Home screen</t>
         </is>
       </c>
     </row>
@@ -3049,20 +3049,74 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
+          <t>Node.js</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>20+ (tested 22.22)</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Developer PC / CI</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>node build.mjs; tests in tests/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Build / test</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Playwright + Chromium</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1.47+</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>End-to-end tests with fake GPS and camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Build / test</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>Azurite</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>3.x</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>CI</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Local Azure Storage emulator for store tests</t>
         </is>

</xml_diff>